<commit_message>
Deploy latest FDA MAUDE Excel report
</commit_message>
<xml_diff>
--- a/fda_maude_apex_2025_2026_iso_summary.xlsx
+++ b/fda_maude_apex_2025_2026_iso_summary.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Carol</t>
+          <t>Regine</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FDA MAUDE Database (2025-01-01 至 2026-09-06)</t>
+          <t>FDA MAUDE Database (至 2026-09-13)</t>
         </is>
       </c>
     </row>

</xml_diff>